<commit_message>
Múltiples correcciones y ratings actualizados
</commit_message>
<xml_diff>
--- a/data/raw/ratings_estatales.xlsx
+++ b/data/raw/ratings_estatales.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Edward\Desktop\Bancomext\Estatales\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Edward\Desktop\Bancomext\Estatales\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E487B902-3352-4765-A505-422EA4AFBEB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C15722A-205F-4078-B17B-2CD8CCE52125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{C54EECCA-873F-4197-AE9F-F2EB0688C0DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Ratings" sheetId="1" r:id="rId1"/>
+    <sheet name="Calificaciones" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,8 +36,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="163">
   <si>
     <t>Clave</t>
   </si>
@@ -429,6 +452,102 @@
   </si>
   <si>
     <t>029</t>
+  </si>
+  <si>
+    <t>Descripción</t>
+  </si>
+  <si>
+    <t>BB</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>BB+</t>
+  </si>
+  <si>
+    <t>BB-</t>
+  </si>
+  <si>
+    <t>B+</t>
+  </si>
+  <si>
+    <t>B-</t>
+  </si>
+  <si>
+    <t>CCC+</t>
+  </si>
+  <si>
+    <t>CCC</t>
+  </si>
+  <si>
+    <t>CCC-</t>
+  </si>
+  <si>
+    <t>CC</t>
+  </si>
+  <si>
+    <t>SD</t>
+  </si>
+  <si>
+    <t>Máxima calidad, mínimo riesgo.</t>
+  </si>
+  <si>
+    <t>Muy alta calidad, muy bajo riesgo.</t>
+  </si>
+  <si>
+    <t>Alta calidad, bajo riesgo.</t>
+  </si>
+  <si>
+    <t>Buena calidad, riesgo moderado.</t>
+  </si>
+  <si>
+    <t>Seguridad aceptable, bajo riesgo.</t>
+  </si>
+  <si>
+    <t>Seguridad moderada, riesgo moderado.</t>
+  </si>
+  <si>
+    <t>Seguridad baja, susceptibles a default.</t>
+  </si>
+  <si>
+    <t>Seguridad insuficiente, alto riesgo.</t>
+  </si>
+  <si>
+    <t>Alta probabilidad de default.</t>
+  </si>
+  <si>
+    <t>En default o altamente probable de estarlo.</t>
+  </si>
+  <si>
+    <t>Especulativo, riesgo sustancial.</t>
+  </si>
+  <si>
+    <t>Altamente especulativo, alto riesgo.</t>
+  </si>
+  <si>
+    <t>Riesgo sustancial, posibilidad real de default.</t>
+  </si>
+  <si>
+    <t>Muy alto riesgo, en default o por ocurrir.</t>
+  </si>
+  <si>
+    <t>Default en comienzo.</t>
+  </si>
+  <si>
+    <t>Emisores ya dejaron de pagar algunas obligaciones.</t>
+  </si>
+  <si>
+    <t>Emisores probablemente no paguen obligaciones, proceso de quiebra.</t>
+  </si>
+  <si>
+    <t>Descripcion</t>
   </si>
 </sst>
 </file>
@@ -807,7 +926,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{764BDB02-0437-47C5-9FBF-8C740C4A6734}">
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.77734375" bestFit="1" customWidth="1"/>
@@ -816,9 +935,10 @@
     <col min="4" max="4" width="15.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="32.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>82</v>
       </c>
@@ -837,8 +957,11 @@
       <c r="F1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>83</v>
       </c>
@@ -857,8 +980,12 @@
       <c r="F2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G2" t="str" cm="1">
+        <f t="array" ref="G2">_xlfn.XLOOKUP(A2&amp;E2,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>83</v>
       </c>
@@ -877,8 +1004,12 @@
       <c r="F3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G3" t="str" cm="1">
+        <f t="array" ref="G3">_xlfn.XLOOKUP(A3&amp;E3,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Seguridad aceptable, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>84</v>
       </c>
@@ -897,8 +1028,12 @@
       <c r="F4" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G4" t="str" cm="1">
+        <f t="array" ref="G4">_xlfn.XLOOKUP(A4&amp;E4,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Alta calidad, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>83</v>
       </c>
@@ -917,8 +1052,12 @@
       <c r="F5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G5" t="str" cm="1">
+        <f t="array" ref="G5">_xlfn.XLOOKUP(A5&amp;E5,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Seguridad aceptable, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>84</v>
       </c>
@@ -937,8 +1076,12 @@
       <c r="F6" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G6" t="str" cm="1">
+        <f t="array" ref="G6">_xlfn.XLOOKUP(A6&amp;E6,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Buena calidad, riesgo moderado.</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>83</v>
       </c>
@@ -957,8 +1100,12 @@
       <c r="F7" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G7" t="str" cm="1">
+        <f t="array" ref="G7">_xlfn.XLOOKUP(A7&amp;E7,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>84</v>
       </c>
@@ -977,8 +1124,12 @@
       <c r="F8" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G8" t="str" cm="1">
+        <f t="array" ref="G8">_xlfn.XLOOKUP(A8&amp;E8,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>83</v>
       </c>
@@ -997,8 +1148,12 @@
       <c r="F9" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G9" t="str" cm="1">
+        <f t="array" ref="G9">_xlfn.XLOOKUP(A9&amp;E9,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>84</v>
       </c>
@@ -1017,8 +1172,12 @@
       <c r="F10" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G10" t="str" cm="1">
+        <f t="array" ref="G10">_xlfn.XLOOKUP(A10&amp;E10,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>83</v>
       </c>
@@ -1037,8 +1196,12 @@
       <c r="F11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G11" t="str" cm="1">
+        <f t="array" ref="G11">_xlfn.XLOOKUP(A11&amp;E11,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Seguridad aceptable, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>84</v>
       </c>
@@ -1057,8 +1220,12 @@
       <c r="F12" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G12" t="str" cm="1">
+        <f t="array" ref="G12">_xlfn.XLOOKUP(A12&amp;E12,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Alta calidad, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>83</v>
       </c>
@@ -1077,8 +1244,12 @@
       <c r="F13" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G13" t="str" cm="1">
+        <f t="array" ref="G13">_xlfn.XLOOKUP(A13&amp;E13,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Máxima calidad, mínimo riesgo.</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>84</v>
       </c>
@@ -1097,8 +1268,12 @@
       <c r="F14" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G14" t="str" cm="1">
+        <f t="array" ref="G14">_xlfn.XLOOKUP(A14&amp;E14,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Máxima calidad, mínimo riesgo.</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>83</v>
       </c>
@@ -1117,8 +1292,12 @@
       <c r="F15" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G15" t="str" cm="1">
+        <f t="array" ref="G15">_xlfn.XLOOKUP(A15&amp;E15,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Seguridad aceptable, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>84</v>
       </c>
@@ -1137,8 +1316,12 @@
       <c r="F16" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G16" t="str" cm="1">
+        <f t="array" ref="G16">_xlfn.XLOOKUP(A16&amp;E16,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Alta calidad, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>83</v>
       </c>
@@ -1157,8 +1340,12 @@
       <c r="F17" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G17" t="str" cm="1">
+        <f t="array" ref="G17">_xlfn.XLOOKUP(A17&amp;E17,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Seguridad moderada, riesgo moderado.</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>84</v>
       </c>
@@ -1177,8 +1364,12 @@
       <c r="F18" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G18" t="str" cm="1">
+        <f t="array" ref="G18">_xlfn.XLOOKUP(A18&amp;E18,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Buena calidad, riesgo moderado.</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>83</v>
       </c>
@@ -1197,8 +1388,12 @@
       <c r="F19" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G19" t="str" cm="1">
+        <f t="array" ref="G19">_xlfn.XLOOKUP(A19&amp;E19,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Seguridad moderada, riesgo moderado.</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>84</v>
       </c>
@@ -1217,8 +1412,12 @@
       <c r="F20" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G20" t="str" cm="1">
+        <f t="array" ref="G20">_xlfn.XLOOKUP(A20&amp;E20,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>84</v>
       </c>
@@ -1237,8 +1436,12 @@
       <c r="F21" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G21" t="str" cm="1">
+        <f t="array" ref="G21">_xlfn.XLOOKUP(A21&amp;E21,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Buena calidad, riesgo moderado.</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>84</v>
       </c>
@@ -1257,8 +1460,12 @@
       <c r="F22" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G22" t="str" cm="1">
+        <f t="array" ref="G22">_xlfn.XLOOKUP(A22&amp;E22,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Buena calidad, riesgo moderado.</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>83</v>
       </c>
@@ -1277,8 +1484,12 @@
       <c r="F23" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G23" t="str" cm="1">
+        <f t="array" ref="G23">_xlfn.XLOOKUP(A23&amp;E23,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>84</v>
       </c>
@@ -1297,8 +1508,12 @@
       <c r="F24" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G24" t="str" cm="1">
+        <f t="array" ref="G24">_xlfn.XLOOKUP(A24&amp;E24,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>83</v>
       </c>
@@ -1317,8 +1532,12 @@
       <c r="F25" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G25" t="str" cm="1">
+        <f t="array" ref="G25">_xlfn.XLOOKUP(A25&amp;E25,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>84</v>
       </c>
@@ -1337,8 +1556,12 @@
       <c r="F26" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G26" t="str" cm="1">
+        <f t="array" ref="G26">_xlfn.XLOOKUP(A26&amp;E26,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Máxima calidad, mínimo riesgo.</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>83</v>
       </c>
@@ -1357,8 +1580,12 @@
       <c r="F27" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G27" t="str" cm="1">
+        <f t="array" ref="G27">_xlfn.XLOOKUP(A27&amp;E27,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Seguridad aceptable, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>84</v>
       </c>
@@ -1377,8 +1604,12 @@
       <c r="F28" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G28" t="str" cm="1">
+        <f t="array" ref="G28">_xlfn.XLOOKUP(A28&amp;E28,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Buena calidad, riesgo moderado.</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>83</v>
       </c>
@@ -1397,8 +1628,12 @@
       <c r="F29" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G29" t="str" cm="1">
+        <f t="array" ref="G29">_xlfn.XLOOKUP(A29&amp;E29,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>84</v>
       </c>
@@ -1417,8 +1652,12 @@
       <c r="F30" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G30" t="str" cm="1">
+        <f t="array" ref="G30">_xlfn.XLOOKUP(A30&amp;E30,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>83</v>
       </c>
@@ -1437,8 +1676,12 @@
       <c r="F31" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G31" t="str" cm="1">
+        <f t="array" ref="G31">_xlfn.XLOOKUP(A31&amp;E31,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Seguridad moderada, riesgo moderado.</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>83</v>
       </c>
@@ -1457,8 +1700,12 @@
       <c r="F32" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G32" t="str" cm="1">
+        <f t="array" ref="G32">_xlfn.XLOOKUP(A32&amp;E32,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Seguridad aceptable, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>84</v>
       </c>
@@ -1477,8 +1724,12 @@
       <c r="F33" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G33" t="str" cm="1">
+        <f t="array" ref="G33">_xlfn.XLOOKUP(A33&amp;E33,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Alta calidad, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>83</v>
       </c>
@@ -1497,8 +1748,12 @@
       <c r="F34" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G34" t="str" cm="1">
+        <f t="array" ref="G34">_xlfn.XLOOKUP(A34&amp;E34,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>84</v>
       </c>
@@ -1517,8 +1772,12 @@
       <c r="F35" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G35" t="str" cm="1">
+        <f t="array" ref="G35">_xlfn.XLOOKUP(A35&amp;E35,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>84</v>
       </c>
@@ -1537,8 +1796,12 @@
       <c r="F36" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G36" t="str" cm="1">
+        <f t="array" ref="G36">_xlfn.XLOOKUP(A36&amp;E36,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>84</v>
       </c>
@@ -1557,8 +1820,12 @@
       <c r="F37" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G37" t="str" cm="1">
+        <f t="array" ref="G37">_xlfn.XLOOKUP(A37&amp;E37,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Máxima calidad, mínimo riesgo.</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>83</v>
       </c>
@@ -1577,8 +1844,12 @@
       <c r="F38" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G38" t="str" cm="1">
+        <f t="array" ref="G38">_xlfn.XLOOKUP(A38&amp;E38,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Seguridad aceptable, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>84</v>
       </c>
@@ -1597,8 +1868,12 @@
       <c r="F39" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G39" t="str" cm="1">
+        <f t="array" ref="G39">_xlfn.XLOOKUP(A39&amp;E39,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Alta calidad, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>83</v>
       </c>
@@ -1617,8 +1892,12 @@
       <c r="F40" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G40" t="str" cm="1">
+        <f t="array" ref="G40">_xlfn.XLOOKUP(A40&amp;E40,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Seguridad aceptable, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>84</v>
       </c>
@@ -1637,8 +1916,12 @@
       <c r="F41" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G41" t="str" cm="1">
+        <f t="array" ref="G41">_xlfn.XLOOKUP(A41&amp;E41,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Alta calidad, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>84</v>
       </c>
@@ -1657,8 +1940,12 @@
       <c r="F42" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G42" t="str" cm="1">
+        <f t="array" ref="G42">_xlfn.XLOOKUP(A42&amp;E42,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>83</v>
       </c>
@@ -1677,8 +1964,12 @@
       <c r="F43" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G43" t="str" cm="1">
+        <f t="array" ref="G43">_xlfn.XLOOKUP(A43&amp;E43,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Seguridad aceptable, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>84</v>
       </c>
@@ -1697,8 +1988,12 @@
       <c r="F44" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G44" t="str" cm="1">
+        <f t="array" ref="G44">_xlfn.XLOOKUP(A44&amp;E44,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Alta calidad, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>83</v>
       </c>
@@ -1717,8 +2012,12 @@
       <c r="F45" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G45" t="str" cm="1">
+        <f t="array" ref="G45">_xlfn.XLOOKUP(A45&amp;E45,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>83</v>
       </c>
@@ -1737,8 +2036,12 @@
       <c r="F46" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G46" t="str" cm="1">
+        <f t="array" ref="G46">_xlfn.XLOOKUP(A46&amp;E46,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Seguridad aceptable, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>84</v>
       </c>
@@ -1757,8 +2060,12 @@
       <c r="F47" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G47" t="str" cm="1">
+        <f t="array" ref="G47">_xlfn.XLOOKUP(A47&amp;E47,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Alta calidad, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>128</v>
       </c>
@@ -1777,8 +2084,12 @@
       <c r="F48" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G48" t="e" cm="1">
+        <f t="array" ref="G48">_xlfn.XLOOKUP(A48&amp;E48,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>83</v>
       </c>
@@ -1797,8 +2108,12 @@
       <c r="F49" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G49" t="str" cm="1">
+        <f t="array" ref="G49">_xlfn.XLOOKUP(A49&amp;E49,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Seguridad aceptable, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>84</v>
       </c>
@@ -1817,8 +2132,12 @@
       <c r="F50" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G50" t="str" cm="1">
+        <f t="array" ref="G50">_xlfn.XLOOKUP(A50&amp;E50,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Alta calidad, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>83</v>
       </c>
@@ -1837,8 +2156,12 @@
       <c r="F51" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G51" t="str" cm="1">
+        <f t="array" ref="G51">_xlfn.XLOOKUP(A51&amp;E51,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>84</v>
       </c>
@@ -1857,8 +2180,12 @@
       <c r="F52" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G52" t="str" cm="1">
+        <f t="array" ref="G52">_xlfn.XLOOKUP(A52&amp;E52,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>83</v>
       </c>
@@ -1877,8 +2204,12 @@
       <c r="F53" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G53" t="str" cm="1">
+        <f t="array" ref="G53">_xlfn.XLOOKUP(A53&amp;E53,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Seguridad aceptable, bajo riesgo.</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>84</v>
       </c>
@@ -1896,6 +2227,10 @@
       </c>
       <c r="F54" t="s">
         <v>7</v>
+      </c>
+      <c r="G54" t="str" cm="1">
+        <f t="array" ref="G54">_xlfn.XLOOKUP(A54&amp;E54,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
+        <v>Muy alta calidad, muy bajo riesgo.</v>
       </c>
     </row>
   </sheetData>
@@ -1905,4 +2240,476 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6C21F93-105B-4924-8C1A-00E3C9FEEDD8}">
+  <dimension ref="A1:C42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>83</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" t="s">
+        <v>109</v>
+      </c>
+      <c r="C9" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B10" t="s">
+        <v>104</v>
+      </c>
+      <c r="C10" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>83</v>
+      </c>
+      <c r="B11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C11" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>83</v>
+      </c>
+      <c r="B12" t="s">
+        <v>136</v>
+      </c>
+      <c r="C12" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>83</v>
+      </c>
+      <c r="B13" t="s">
+        <v>132</v>
+      </c>
+      <c r="C13" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>83</v>
+      </c>
+      <c r="B14" t="s">
+        <v>137</v>
+      </c>
+      <c r="C14" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" t="s">
+        <v>138</v>
+      </c>
+      <c r="C15" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" t="s">
+        <v>133</v>
+      </c>
+      <c r="C16" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>83</v>
+      </c>
+      <c r="B17" t="s">
+        <v>139</v>
+      </c>
+      <c r="C17" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>83</v>
+      </c>
+      <c r="B18" t="s">
+        <v>134</v>
+      </c>
+      <c r="C18" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>83</v>
+      </c>
+      <c r="B19" t="s">
+        <v>135</v>
+      </c>
+      <c r="C19" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" t="s">
+        <v>89</v>
+      </c>
+      <c r="C21" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>84</v>
+      </c>
+      <c r="B22" t="s">
+        <v>93</v>
+      </c>
+      <c r="C22" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" t="s">
+        <v>96</v>
+      </c>
+      <c r="C23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>84</v>
+      </c>
+      <c r="B24" t="s">
+        <v>114</v>
+      </c>
+      <c r="C24" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>84</v>
+      </c>
+      <c r="B25" t="s">
+        <v>101</v>
+      </c>
+      <c r="C25" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>84</v>
+      </c>
+      <c r="B26" t="s">
+        <v>85</v>
+      </c>
+      <c r="C26" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>84</v>
+      </c>
+      <c r="B27" t="s">
+        <v>109</v>
+      </c>
+      <c r="C27" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>84</v>
+      </c>
+      <c r="B28" t="s">
+        <v>104</v>
+      </c>
+      <c r="C28" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>84</v>
+      </c>
+      <c r="B29" t="s">
+        <v>106</v>
+      </c>
+      <c r="C29" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>84</v>
+      </c>
+      <c r="B30" t="s">
+        <v>136</v>
+      </c>
+      <c r="C30" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>84</v>
+      </c>
+      <c r="B31" t="s">
+        <v>132</v>
+      </c>
+      <c r="C31" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>84</v>
+      </c>
+      <c r="B32" t="s">
+        <v>137</v>
+      </c>
+      <c r="C32" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>84</v>
+      </c>
+      <c r="B33" t="s">
+        <v>138</v>
+      </c>
+      <c r="C33" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>84</v>
+      </c>
+      <c r="B34" t="s">
+        <v>133</v>
+      </c>
+      <c r="C34" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>84</v>
+      </c>
+      <c r="B35" t="s">
+        <v>139</v>
+      </c>
+      <c r="C35" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>84</v>
+      </c>
+      <c r="B36" t="s">
+        <v>140</v>
+      </c>
+      <c r="C36" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>84</v>
+      </c>
+      <c r="B37" t="s">
+        <v>141</v>
+      </c>
+      <c r="C37" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>84</v>
+      </c>
+      <c r="B38" t="s">
+        <v>142</v>
+      </c>
+      <c r="C38" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>84</v>
+      </c>
+      <c r="B39" t="s">
+        <v>143</v>
+      </c>
+      <c r="C39" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>84</v>
+      </c>
+      <c r="B40" t="s">
+        <v>134</v>
+      </c>
+      <c r="C40" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>84</v>
+      </c>
+      <c r="B41" t="s">
+        <v>144</v>
+      </c>
+      <c r="C41" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>84</v>
+      </c>
+      <c r="B42" t="s">
+        <v>135</v>
+      </c>
+      <c r="C42" t="s">
+        <v>161</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
IMSS junio y nuevos ratings
</commit_message>
<xml_diff>
--- a/data/raw/ratings_estatales.xlsx
+++ b/data/raw/ratings_estatales.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\victo\Documents\BANCOMEXT\HRRatings_Fitch\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\victo\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EA8E4A7-D713-4C0A-87FE-F715806AFF6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{625B3BFD-CC3A-44AA-9D89-6F940EE34604}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{C54EECCA-873F-4197-AE9F-F2EB0688C0DB}"/>
   </bookViews>
@@ -798,7 +798,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{764BDB02-0437-47C5-9FBF-8C740C4A6734}">
-  <sheetPr codeName="Hoja1"/>
+  <sheetPr codeName="Hoja1" filterMode="1"/>
   <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -882,7 +882,7 @@
         <v>Seguridad aceptable, bajo riesgo.</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -930,7 +930,7 @@
         <v>Seguridad aceptable, bajo riesgo.</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>59</v>
       </c>
@@ -965,7 +965,7 @@
         <v>12</v>
       </c>
       <c r="D7" s="2">
-        <v>45803</v>
+        <v>46171</v>
       </c>
       <c r="E7" t="s">
         <v>63</v>
@@ -978,7 +978,7 @@
         <v>Muy alta calidad, muy bajo riesgo.</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>59</v>
       </c>
@@ -1026,7 +1026,7 @@
         <v>Muy alta calidad, muy bajo riesgo.</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -1037,7 +1037,7 @@
         <v>14</v>
       </c>
       <c r="D10" s="2">
-        <v>45835</v>
+        <v>46199</v>
       </c>
       <c r="E10" t="s">
         <v>68</v>
@@ -1074,7 +1074,7 @@
         <v>Seguridad aceptable, bajo riesgo.</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>59</v>
       </c>
@@ -1122,7 +1122,7 @@
         <v>Máxima calidad, mínimo riesgo.</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>59</v>
       </c>
@@ -1170,7 +1170,7 @@
         <v>Seguridad aceptable, bajo riesgo.</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>59</v>
       </c>
@@ -1181,13 +1181,13 @@
         <v>21</v>
       </c>
       <c r="D16" s="2">
-        <v>45799</v>
+        <v>46162</v>
       </c>
       <c r="E16" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="F16" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="G16" t="str" cm="1">
         <f t="array" ref="G16">_xlfn.XLOOKUP(A16&amp;E16,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
@@ -1218,7 +1218,7 @@
         <v>Seguridad moderada, riesgo moderado.</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>59</v>
       </c>
@@ -1266,7 +1266,7 @@
         <v>Seguridad moderada, riesgo moderado.</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>59</v>
       </c>
@@ -1290,7 +1290,7 @@
         <v>Muy alta calidad, muy bajo riesgo.</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>59</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>Máxima calidad, mínimo riesgo.</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>59</v>
       </c>
@@ -1362,7 +1362,7 @@
         <v>Muy alta calidad, muy bajo riesgo.</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>59</v>
       </c>
@@ -1373,7 +1373,7 @@
         <v>29</v>
       </c>
       <c r="D24" s="2">
-        <v>45799</v>
+        <v>46157</v>
       </c>
       <c r="E24" t="s">
         <v>63</v>
@@ -1410,7 +1410,7 @@
         <v>Muy alta calidad, muy bajo riesgo.</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>59</v>
       </c>
@@ -1458,7 +1458,7 @@
         <v>Seguridad aceptable, bajo riesgo.</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>59</v>
       </c>
@@ -1493,20 +1493,20 @@
         <v>33</v>
       </c>
       <c r="D29" s="2">
-        <v>45828</v>
+        <v>46198</v>
       </c>
       <c r="E29" t="s">
         <v>68</v>
       </c>
       <c r="F29" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="G29" t="str" cm="1">
         <f t="array" ref="G29">_xlfn.XLOOKUP(A29&amp;E29,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
         <v>Muy alta calidad, muy bajo riesgo.</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>59</v>
       </c>
@@ -1517,7 +1517,7 @@
         <v>33</v>
       </c>
       <c r="D30" s="2">
-        <v>45818</v>
+        <v>46182</v>
       </c>
       <c r="E30" t="s">
         <v>68</v>
@@ -1578,7 +1578,7 @@
         <v>Seguridad aceptable, bajo riesgo.</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>59</v>
       </c>
@@ -1589,10 +1589,10 @@
         <v>37</v>
       </c>
       <c r="D33" s="2">
-        <v>45799</v>
+        <v>46162</v>
       </c>
       <c r="E33" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="F33" t="s">
         <v>67</v>
@@ -1626,7 +1626,7 @@
         <v>Muy alta calidad, muy bajo riesgo.</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>59</v>
       </c>
@@ -1650,7 +1650,7 @@
         <v>Muy alta calidad, muy bajo riesgo.</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>59</v>
       </c>
@@ -1674,7 +1674,7 @@
         <v>Muy alta calidad, muy bajo riesgo.</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>59</v>
       </c>
@@ -1722,7 +1722,7 @@
         <v>Seguridad aceptable, bajo riesgo.</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>59</v>
       </c>
@@ -1733,13 +1733,13 @@
         <v>41</v>
       </c>
       <c r="D39" s="2">
-        <v>45818</v>
+        <v>46182</v>
       </c>
       <c r="E39" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="F39" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="G39" t="str" cm="1">
         <f t="array" ref="G39">_xlfn.XLOOKUP(A39&amp;E39,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
@@ -1757,20 +1757,20 @@
         <v>43</v>
       </c>
       <c r="D40" s="2">
-        <v>45807</v>
+        <v>45809</v>
       </c>
       <c r="E40" t="s">
         <v>71</v>
       </c>
       <c r="F40" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="G40" t="str" cm="1">
         <f t="array" ref="G40">_xlfn.XLOOKUP(A40&amp;E40,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
         <v>Seguridad aceptable, bajo riesgo.</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>59</v>
       </c>
@@ -1794,7 +1794,7 @@
         <v>Alta calidad, bajo riesgo.</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>59</v>
       </c>
@@ -1842,7 +1842,7 @@
         <v>Seguridad aceptable, bajo riesgo.</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>59</v>
       </c>
@@ -1914,7 +1914,7 @@
         <v>Seguridad aceptable, bajo riesgo.</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>59</v>
       </c>
@@ -1938,7 +1938,7 @@
         <v>Alta calidad, bajo riesgo.</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>83</v>
       </c>
@@ -1986,7 +1986,7 @@
         <v>Seguridad aceptable, bajo riesgo.</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>59</v>
       </c>
@@ -2034,7 +2034,7 @@
         <v>Muy alta calidad, muy bajo riesgo.</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>59</v>
       </c>
@@ -2051,7 +2051,7 @@
         <v>68</v>
       </c>
       <c r="F52" t="s">
-        <v>6</v>
+        <v>67</v>
       </c>
       <c r="G52" t="str" cm="1">
         <f t="array" ref="G52">_xlfn.XLOOKUP(A52&amp;E52,Calificaciones!$A$2:$A$42 &amp; Calificaciones!$B$2:$B$42,Calificaciones!$C$2:$C$42)</f>
@@ -2082,7 +2082,7 @@
         <v>Seguridad aceptable, bajo riesgo.</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>59</v>
       </c>
@@ -2107,6 +2107,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G54" xr:uid="{764BDB02-0437-47C5-9FBF-8C740C4A6734}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="HR"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F54">
     <sortCondition ref="C2:C54"/>
   </sortState>

</xml_diff>